<commit_message>
added irt material to processor
</commit_message>
<xml_diff>
--- a/cubes/data/materials/materials.xlsx
+++ b/cubes/data/materials/materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannes/Work/CUBES/cubes/data/materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/SSK Harddrive/CUBES/cubes/data/materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5134A9C7-6310-9C4C-9846-89EBF64D6E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA4F513-56CA-F640-92B5-A6CF1DB275C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="560" yWindow="-15800" windowWidth="26660" windowHeight="15800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="860" windowWidth="19200" windowHeight="22220" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="115">
   <si>
     <t>Material</t>
   </si>
@@ -339,6 +339,48 @@
   </si>
   <si>
     <t>Adiabatic_insulation</t>
+  </si>
+  <si>
+    <t>beizaee_brick_outer_leaf</t>
+  </si>
+  <si>
+    <t>beizaee_brick_inner_leaf</t>
+  </si>
+  <si>
+    <t>beizaee_plaster_dense</t>
+  </si>
+  <si>
+    <t>beizaee_clay_tile</t>
+  </si>
+  <si>
+    <t>beizaee_roofing_felt</t>
+  </si>
+  <si>
+    <t>beizaee_polyisocyanurate</t>
+  </si>
+  <si>
+    <t>beizaee_timber_flooring</t>
+  </si>
+  <si>
+    <t>beizaee_cast_concrete</t>
+  </si>
+  <si>
+    <t>beizaee_carpet</t>
+  </si>
+  <si>
+    <t>beizaee_plasterboard</t>
+  </si>
+  <si>
+    <t>beizaee_painted_oak</t>
+  </si>
+  <si>
+    <t>InfraredTransparent</t>
+  </si>
+  <si>
+    <t>IRTMaterial</t>
+  </si>
+  <si>
+    <t>Door_WoodSolid_35mm</t>
   </si>
 </sst>
 </file>
@@ -421,9 +463,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -461,7 +503,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -567,7 +609,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -709,7 +751,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -717,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -728,7 +770,7 @@
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -762,8 +804,11 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -797,8 +842,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -836,8 +884,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -875,8 +926,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -914,8 +968,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -953,8 +1010,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -992,8 +1052,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1031,8 +1094,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1070,8 +1136,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1109,8 +1178,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1148,8 +1220,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1187,8 +1262,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -1226,8 +1304,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1265,8 +1346,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1304,8 +1388,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -1343,8 +1430,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1382,8 +1472,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1421,8 +1514,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1460,8 +1556,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1499,8 +1598,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1538,8 +1640,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1573,8 +1678,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -1612,8 +1720,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>34</v>
       </c>
@@ -1651,8 +1762,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -1690,8 +1804,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1729,8 +1846,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1768,8 +1888,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -1807,8 +1930,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -1846,8 +1972,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -1885,8 +2014,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -1924,8 +2056,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -1952,8 +2087,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -1980,8 +2118,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -2008,8 +2149,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>46</v>
       </c>
@@ -2036,8 +2180,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -2067,8 +2214,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -2102,8 +2252,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -2137,8 +2290,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -2172,8 +2328,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L39" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -2203,8 +2362,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>52</v>
       </c>
@@ -2238,8 +2400,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>53</v>
       </c>
@@ -2273,8 +2438,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -2292,8 +2460,11 @@
         <f>TRUE()</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>54</v>
       </c>
@@ -2327,8 +2498,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -2346,8 +2520,11 @@
         <f>TRUE()</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>55</v>
       </c>
@@ -2381,8 +2558,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>56</v>
       </c>
@@ -2416,8 +2596,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>57</v>
       </c>
@@ -2451,8 +2634,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>59</v>
       </c>
@@ -2479,8 +2665,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L49" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>60</v>
       </c>
@@ -2505,8 +2694,11 @@
       <c r="K50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L50" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>61</v>
       </c>
@@ -2531,8 +2723,11 @@
       <c r="K51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>62</v>
       </c>
@@ -2565,8 +2760,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>63</v>
       </c>
@@ -2599,8 +2797,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>64</v>
       </c>
@@ -2633,8 +2834,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>65</v>
       </c>
@@ -2667,8 +2871,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>66</v>
       </c>
@@ -2701,8 +2908,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>67</v>
       </c>
@@ -2735,8 +2945,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>68</v>
       </c>
@@ -2769,8 +2982,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>69</v>
       </c>
@@ -2803,8 +3019,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>70</v>
       </c>
@@ -2837,8 +3056,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>71</v>
       </c>
@@ -2871,8 +3093,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>72</v>
       </c>
@@ -2905,8 +3130,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>73</v>
       </c>
@@ -2939,8 +3167,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>74</v>
       </c>
@@ -2973,8 +3204,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -3007,8 +3241,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>76</v>
       </c>
@@ -3041,8 +3278,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>77</v>
       </c>
@@ -3075,8 +3315,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>78</v>
       </c>
@@ -3109,8 +3352,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -3143,8 +3389,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L69" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>80</v>
       </c>
@@ -3177,8 +3426,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L70" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>81</v>
       </c>
@@ -3211,8 +3463,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>82</v>
       </c>
@@ -3245,8 +3500,11 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L72" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -3277,8 +3535,11 @@
       <c r="K73" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L73" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>84</v>
       </c>
@@ -3309,8 +3570,11 @@
       <c r="K74" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L74" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>85</v>
       </c>
@@ -3341,8 +3605,11 @@
       <c r="K75" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>86</v>
       </c>
@@ -3373,8 +3640,11 @@
       <c r="K76" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L76" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>87</v>
       </c>
@@ -3399,8 +3669,11 @@
       <c r="K77" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L77" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>88</v>
       </c>
@@ -3431,8 +3704,11 @@
       <c r="K78" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L78" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>89</v>
       </c>
@@ -3463,8 +3739,11 @@
       <c r="K79" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L79" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>90</v>
       </c>
@@ -3495,8 +3774,11 @@
       <c r="K80" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>91</v>
       </c>
@@ -3527,8 +3809,11 @@
       <c r="K81" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L81" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>92</v>
       </c>
@@ -3559,8 +3844,11 @@
       <c r="K82" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L82" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>98</v>
       </c>
@@ -3591,8 +3879,11 @@
       <c r="K83" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L83" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>97</v>
       </c>
@@ -3623,8 +3914,11 @@
       <c r="K84" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L84" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>93</v>
       </c>
@@ -3649,8 +3943,11 @@
       <c r="K85" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L85" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>94</v>
       </c>
@@ -3681,8 +3978,11 @@
       <c r="K86" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L86" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>96</v>
       </c>
@@ -3713,8 +4013,11 @@
       <c r="K87" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L87" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>95</v>
       </c>
@@ -3745,8 +4048,11 @@
       <c r="K88" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L88" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>99</v>
       </c>
@@ -3777,8 +4083,11 @@
       <c r="K89" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L89" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>100</v>
       </c>
@@ -3808,6 +4117,437 @@
       </c>
       <c r="K90" t="b">
         <v>0</v>
+      </c>
+      <c r="L90" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>101</v>
+      </c>
+      <c r="B91">
+        <v>0.84</v>
+      </c>
+      <c r="D91">
+        <v>800</v>
+      </c>
+      <c r="E91">
+        <v>1700</v>
+      </c>
+      <c r="F91" t="s">
+        <v>12</v>
+      </c>
+      <c r="G91">
+        <v>0.9</v>
+      </c>
+      <c r="H91">
+        <v>0.7</v>
+      </c>
+      <c r="I91">
+        <v>0.7</v>
+      </c>
+      <c r="J91" t="b">
+        <v>0</v>
+      </c>
+      <c r="K91" t="b">
+        <v>0</v>
+      </c>
+      <c r="L91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>102</v>
+      </c>
+      <c r="B92">
+        <v>0.62</v>
+      </c>
+      <c r="D92">
+        <v>800</v>
+      </c>
+      <c r="E92">
+        <v>1700</v>
+      </c>
+      <c r="F92" t="s">
+        <v>12</v>
+      </c>
+      <c r="G92">
+        <v>0.9</v>
+      </c>
+      <c r="H92">
+        <v>0.7</v>
+      </c>
+      <c r="I92">
+        <v>0.7</v>
+      </c>
+      <c r="J92" t="b">
+        <v>0</v>
+      </c>
+      <c r="K92" t="b">
+        <v>0</v>
+      </c>
+      <c r="L92" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>103</v>
+      </c>
+      <c r="B93">
+        <v>0.5</v>
+      </c>
+      <c r="D93">
+        <v>1000</v>
+      </c>
+      <c r="E93">
+        <v>1300</v>
+      </c>
+      <c r="F93" t="s">
+        <v>58</v>
+      </c>
+      <c r="G93">
+        <v>0.9</v>
+      </c>
+      <c r="H93">
+        <v>0.7</v>
+      </c>
+      <c r="I93">
+        <v>0.7</v>
+      </c>
+      <c r="J93" t="b">
+        <v>0</v>
+      </c>
+      <c r="K93" t="b">
+        <v>0</v>
+      </c>
+      <c r="L93" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>104</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="D94">
+        <v>800</v>
+      </c>
+      <c r="E94">
+        <v>2000</v>
+      </c>
+      <c r="F94" t="s">
+        <v>47</v>
+      </c>
+      <c r="G94">
+        <v>0.9</v>
+      </c>
+      <c r="H94">
+        <v>0.7</v>
+      </c>
+      <c r="I94">
+        <v>0.7</v>
+      </c>
+      <c r="J94" t="b">
+        <v>0</v>
+      </c>
+      <c r="K94" t="b">
+        <v>0</v>
+      </c>
+      <c r="L94" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>105</v>
+      </c>
+      <c r="B95">
+        <v>0.19</v>
+      </c>
+      <c r="D95">
+        <v>837</v>
+      </c>
+      <c r="E95">
+        <v>960</v>
+      </c>
+      <c r="F95" t="s">
+        <v>12</v>
+      </c>
+      <c r="G95">
+        <v>0.9</v>
+      </c>
+      <c r="H95">
+        <v>0.7</v>
+      </c>
+      <c r="I95">
+        <v>0.7</v>
+      </c>
+      <c r="J95" t="b">
+        <v>0</v>
+      </c>
+      <c r="K95" t="b">
+        <v>0</v>
+      </c>
+      <c r="L95" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>106</v>
+      </c>
+      <c r="B96">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="D96">
+        <v>1470</v>
+      </c>
+      <c r="E96">
+        <v>45</v>
+      </c>
+      <c r="F96" t="s">
+        <v>12</v>
+      </c>
+      <c r="G96">
+        <v>0.9</v>
+      </c>
+      <c r="H96">
+        <v>0.7</v>
+      </c>
+      <c r="I96">
+        <v>0.7</v>
+      </c>
+      <c r="J96" t="b">
+        <v>0</v>
+      </c>
+      <c r="K96" t="b">
+        <v>0</v>
+      </c>
+      <c r="L96" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>107</v>
+      </c>
+      <c r="B97">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="D97">
+        <v>1200</v>
+      </c>
+      <c r="E97">
+        <v>650</v>
+      </c>
+      <c r="F97" t="s">
+        <v>47</v>
+      </c>
+      <c r="G97">
+        <v>0.9</v>
+      </c>
+      <c r="H97">
+        <v>0.7</v>
+      </c>
+      <c r="I97">
+        <v>0.7</v>
+      </c>
+      <c r="J97" t="b">
+        <v>0</v>
+      </c>
+      <c r="K97" t="b">
+        <v>0</v>
+      </c>
+      <c r="L97" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>108</v>
+      </c>
+      <c r="B98">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="D98">
+        <v>1000</v>
+      </c>
+      <c r="E98">
+        <v>2000</v>
+      </c>
+      <c r="F98" t="s">
+        <v>12</v>
+      </c>
+      <c r="G98">
+        <v>0.9</v>
+      </c>
+      <c r="H98">
+        <v>0.7</v>
+      </c>
+      <c r="I98">
+        <v>0.7</v>
+      </c>
+      <c r="J98" t="b">
+        <v>0</v>
+      </c>
+      <c r="K98" t="b">
+        <v>0</v>
+      </c>
+      <c r="L98" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>109</v>
+      </c>
+      <c r="B99">
+        <v>0.06</v>
+      </c>
+      <c r="D99">
+        <v>1300</v>
+      </c>
+      <c r="E99">
+        <v>200</v>
+      </c>
+      <c r="F99" t="s">
+        <v>12</v>
+      </c>
+      <c r="G99">
+        <v>0.95</v>
+      </c>
+      <c r="H99">
+        <v>0.7</v>
+      </c>
+      <c r="I99">
+        <v>0.7</v>
+      </c>
+      <c r="J99" t="b">
+        <v>0</v>
+      </c>
+      <c r="K99" t="b">
+        <v>0</v>
+      </c>
+      <c r="L99" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>110</v>
+      </c>
+      <c r="B100">
+        <v>0.25</v>
+      </c>
+      <c r="D100">
+        <v>896</v>
+      </c>
+      <c r="E100">
+        <v>2800</v>
+      </c>
+      <c r="F100" t="s">
+        <v>58</v>
+      </c>
+      <c r="G100">
+        <v>0.9</v>
+      </c>
+      <c r="H100">
+        <v>0.7</v>
+      </c>
+      <c r="I100">
+        <v>0.7</v>
+      </c>
+      <c r="J100" t="b">
+        <v>0</v>
+      </c>
+      <c r="K100" t="b">
+        <v>0</v>
+      </c>
+      <c r="L100" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>111</v>
+      </c>
+      <c r="B101">
+        <v>0.19</v>
+      </c>
+      <c r="D101">
+        <v>2390</v>
+      </c>
+      <c r="E101">
+        <v>700</v>
+      </c>
+      <c r="F101" t="s">
+        <v>58</v>
+      </c>
+      <c r="G101">
+        <v>0.9</v>
+      </c>
+      <c r="H101">
+        <v>0.7</v>
+      </c>
+      <c r="I101">
+        <v>0.7</v>
+      </c>
+      <c r="J101" t="b">
+        <v>0</v>
+      </c>
+      <c r="K101" t="b">
+        <v>0</v>
+      </c>
+      <c r="L101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>114</v>
+      </c>
+      <c r="B102">
+        <v>0.19</v>
+      </c>
+      <c r="D102">
+        <v>700</v>
+      </c>
+      <c r="E102">
+        <v>2390</v>
+      </c>
+      <c r="F102" t="s">
+        <v>12</v>
+      </c>
+      <c r="G102">
+        <v>0.9</v>
+      </c>
+      <c r="H102">
+        <v>0.5</v>
+      </c>
+      <c r="I102">
+        <v>0.5</v>
+      </c>
+      <c r="J102" t="b">
+        <v>0</v>
+      </c>
+      <c r="K102" t="b">
+        <v>0</v>
+      </c>
+      <c r="L102" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>113</v>
+      </c>
+      <c r="L103" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>